<commit_message>
PCB makinesi BOM: hot plate icin EMS 500 W plaka rezistans (2.424,47 TL)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XTzihDN3mirVxqDnEvzLhN
</commit_message>
<xml_diff>
--- a/pcb-makinesi/bom-v0.xlsx
+++ b/pcb-makinesi/bom-v0.xlsx
@@ -4490,7 +4490,7 @@
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>PTC alüminyum 220 V 600 W ~260 °C (ya da silikon ped + 6 mm Al plaka)</t>
+          <t>500 W plaka rezistans, 220 V (ölçü teyit edilecek; hedef ~200x150 mm)</t>
         </is>
       </c>
       <c r="E57" s="2" t="n">
@@ -4501,21 +4501,19 @@
           <t>adet</t>
         </is>
       </c>
-      <c r="G57" s="3" t="n"/>
+      <c r="G57" s="3" t="n">
+        <v>2424.47</v>
+      </c>
       <c r="H57" s="3">
         <f>IF(G57="","",E57*G57)</f>
         <v/>
       </c>
       <c r="I57" s="6" t="inlineStr">
         <is>
-          <t>Amazon.com.tr (Hyuduo)</t>
-        </is>
-      </c>
-      <c r="J57" s="8" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com.tr/Hyuduo-istasyonu-lehimleme-plakas%C4%B1-%C3%A7%C4%B1kar%C4%B1c%C4%B1/dp/B09P3RP4ZJ</t>
-        </is>
-      </c>
+          <t>EMS Endüstriyel</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr"/>
       <c r="K57" s="6" t="inlineStr">
         <is>
           <t>?</t>
@@ -4528,7 +4526,7 @@
       </c>
       <c r="M57" s="6" t="inlineStr">
         <is>
-          <t>Elektronik mağazalarında yok. Ürün için ~200x150 mm 500 W döküm/plaka rezistans teklifi al. Hazır alt.: Sunline 958 130x130, Robotistan 13.145,64 TL (Alternatifler).</t>
+          <t>Fiyatı kullanıcı buldu (2026-10-04); link/ölçü eklenecek. Üstüne 6 mm alüminyum plaka + termokupl. Hazır alt.: Sunline 958 130x130, Robotistan 13.145,64 TL (Alternatifler).</t>
         </is>
       </c>
     </row>
@@ -5922,30 +5920,29 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J56" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J58" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J59" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J60" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J63" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J64" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J65" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J66" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J67" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J68" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J69" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J71" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J72" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J73" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J74" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J75" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J77" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J78" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J79" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J58" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J59" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J60" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J63" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J64" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J65" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J66" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J67" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J68" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J69" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J71" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J72" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J73" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J74" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J75" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J77" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J78" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J79" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J80" r:id="rId78"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
PCB delme makinesi v0: parametrik tasarim (gen_delme.py)
Sabit spindle + capraz tabla (Y alt, X ust), 28BYJ-48 + baski GT2-20 kasnak,
Z = 28BYJ + T8, 775 + JT0 spindle. 160x100 hareket (Eurocard), 6.6" ekranin
143x90 desen alani icinde; hizalama pimleri x=±76. Betik 18 uc konumda parca
cakismasini denetler; STL'ler, 3 gorunus cizimi, olculer.txt ve kaydirmali 3B
onizleme (onizleme.html) uretir. BOM: ana panel Aptus 6.6" 4K.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XTzihDN3mirVxqDnEvzLhN
</commit_message>
<xml_diff>
--- a/pcb-makinesi/bom-v0.xlsx
+++ b/pcb-makinesi/bom-v0.xlsx
@@ -1231,12 +1231,12 @@
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>Mono LCD 10.3" 8K (Aptus)</t>
+          <t>Mono LCD 6.6" 4K (Aptus)</t>
         </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
-          <t>Aptus DBM103M8K01, 7680x4320, ~30 µm, ~228x128 mm (hesap), LTPS, MIPI 50 pin</t>
+          <t>Aptus DBM066M4K01, 4098x2560, 35 µm, aktif alan 143.43x89.60 mm, MIPI 50 pin (master+slave)</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="J2" s="8" t="inlineStr">
         <is>
-          <t>https://www.aptusdisplay.com/products/10-3-inch-8k-7680x4320-mipi-50pin-mono-lcd-screen</t>
+          <t>https://www.aptusdisplay.com/products/6-6-inch-4k-4098x2560-mono-lcd-display</t>
         </is>
       </c>
       <c r="K2" s="6" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="M2" s="6" t="inlineStr">
         <is>
-          <t>Üretici kaynağı (yedek parça değil). Fiyat, MOQ, 405 nm geçirgenlik, UV ömrü, cam kalınlığı sorulacak (e-posta taslağı hazır). 150x100 kartı kapsar.</t>
+          <t>Kullanıcının seçimi (2026-10-04). Desen ≤143x89 mm; ham plaket 160x100, hizalama pimleri kenarda (delme makinesiyle aynı). Fiyat/MOQ/405 nm geçirgenlik sorulacak.</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="J3" s="8" t="inlineStr">
         <is>
-          <t>https://www.aptusdisplay.com/products/10-3-inch-8k-7680x4320-mipi-50pin-mono-lcd-screen</t>
+          <t>https://www.aptusdisplay.com/products/6-6-inch-4k-4098x2560-mono-lcd-display</t>
         </is>
       </c>
       <c r="K3" s="6" t="inlineStr">
@@ -1332,7 +1332,7 @@
       </c>
       <c r="M3" s="6" t="inlineStr">
         <is>
-          <t>Panel MIPI zamanlamasını çözmeden HDMI ile sürülür. Giriş çözünürlüğü/EDID ve mono piksel paketlemesi sorulacak.</t>
+          <t>Panel MIPI zamanlamasını çözmeden HDMI ile sürülür (6.6" panel için). Giriş çözünürlüğü/EDID ve mono piksel paketlemesi sorulacak.</t>
         </is>
       </c>
     </row>
@@ -6017,12 +6017,12 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Aptus 6.6" 4K mono LCD</t>
+          <t>Aptus 10.3" 8K mono LCD</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>DBM066M4K01, 4098x2560, 35 µm, aktif alan 143.43x89.60 mm, MIPI 50 pin (master+slave)</t>
+          <t>DBM103M8K01, 7680x4320, ~30 µm, ~228x128 mm (hesap), MIPI 50 pin</t>
         </is>
       </c>
       <c r="D2" s="3" t="n"/>
@@ -6033,7 +6033,7 @@
       </c>
       <c r="F2" s="8" t="inlineStr">
         <is>
-          <t>https://www.aptusdisplay.com/products/6-6-inch-4k-4098x2560-mono-lcd-display</t>
+          <t>https://www.aptusdisplay.com/products/10-3-inch-8k-7680x4320-mipi-50pin-mono-lcd-screen</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -6043,7 +6043,7 @@
       </c>
       <c r="H2" s="6" t="inlineStr">
         <is>
-          <t>Daha ucuz/yaygın boy ama 150x100 kart SIĞMAZ (en büyük kart ~140x85). HDMI kartı var.</t>
+          <t>Daha büyük kartlar (150x100 desen) gerekirse.</t>
         </is>
       </c>
     </row>
@@ -6988,7 +6988,7 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Aptus 10.3" 8K mono LCD + HDMI→MIPI kartı</t>
+          <t>Aptus 6.6" 4K mono LCD + HDMI→MIPI kartı</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">

</xml_diff>

<commit_message>
PCB delme makinesi: fiyatli parca listesi (BOM sayfasi, ~3.400 TL)
Turkiye fiyatlari (2026-10-04): 28BYJ RobitShop 54 TL, LM8UU 42, 300 mm krom
mil (250 yok), hazir disli olmayan GT2 avara (623ZZ yok), RS775 + 5 mm pens
seti (MAN02 3,175 sapi tutmaz), T8x8 400 mm. README buna gore guncellendi.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XTzihDN3mirVxqDnEvzLhN
</commit_message>
<xml_diff>
--- a/pcb-makinesi/bom-v0.xlsx
+++ b/pcb-makinesi/bom-v0.xlsx
@@ -9,13 +9,14 @@
   <sheets>
     <sheet name="Özet" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Kesim karşılaştırma" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="BOM" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Alternatifler" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Yurt dışı" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Uyarılar" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Delme makinesi v0" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="BOM" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Alternatifler" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Yurt dışı" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Uyarılar" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'BOM'!$A$1:$M$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'BOM'!$A$1:$M$80</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1135,6 +1136,975 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="56" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Kalem</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Özellik</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Birim fiyat (TL)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Toplam (TL)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Satıcı</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Stok</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Doğrulandı</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Not</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>28BYJ-48 5 V + ULN2003</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>X, Y, Z eksenleri</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>54.05</v>
+      </c>
+      <c r="E2" s="3">
+        <f>IF(D2="","",C2*D2)</f>
+        <v/>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>RobitShop</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>https://www.robitshop.com/urun/28-byj-48-reduktorlu-step-motor-ve-uln2003-step-motor-surucu-karti-mavi</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Var (397)</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>evet</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>Alt.: Direnc 92,99, Robotistan 100,98. 12 V sürümü TR'de yok.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>LM8UU</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>8 mm lineer rulman (X 4, Y 4, Z 4)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="E3" s="3">
+        <f>IF(D3="","",C3*D3)</f>
+        <v/>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Motorobit</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>https://www.motorobit.com/3d-yazici-icin-rulman-lm8uu</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Var (75)</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>evet</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Krom mil Ø8, 300 mm</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Kes: X 2x262, Y 2x250, Z 2x110 (bir milden)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>138</v>
+      </c>
+      <c r="E4" s="3">
+        <f>IF(D4="","",C4*D4)</f>
+        <v/>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Motorobit</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>https://www.motorobit.com/8mm-induksiyonlu-mil-krom-kapli-300mm</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Var (26)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>evet</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>250/330 mm TR'de yok. Sertleştirilmiş mil taşla (avuç taşlama) kesilir; yerel lineer rulmancıda kestirmek daha ucuz olabilir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>GT2 kayış 6 mm, 2 m</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>X 620 + Y 596 mm</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>116.24</v>
+      </c>
+      <c r="E5" s="3">
+        <f>IF(D5="","",C5*D5)</f>
+        <v/>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Direnc.net</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>https://www.direnc.net/gt2-zamanlama-kayisi-6mm-2-metre</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Var (22)</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>evet</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>1 m yetmez.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>GT2 dişsiz rulmanlı avara (3 mm)</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Hazır avara; baskı avara yerine</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>66</v>
+      </c>
+      <c r="E6" s="3">
+        <f>IF(D6="","",C6*D6)</f>
+        <v/>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Motorobit</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>https://www.motorobit.com/gt2-dissiz-3mm-rulmanli-kasnak</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Var (524)</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>evet</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>623ZZ TR'de bulunamadı (624ZZ baskı avaraya sığmaz). Baskı kasnaklar yine 28BYJ miline (D 5/3 mm).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>RS775 DC motor, 5 mm mil</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>12–36 V, rulmanlı, "3000 rpm"</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>270.22</v>
+      </c>
+      <c r="E7" s="3">
+        <f>IF(D7="","",C7*D7)</f>
+        <v/>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>RobitShop</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>https://www.robitshop.com/urun/rs775-dc-motor-rulmanli-12v-3000-rpm-sarjli-matkap-motoru</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Var (12)</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>evet</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>PCB için devir düşük (karbür ~10.000 rpm sever): yavaş ilerle ya da daha hızlı 775 bul (pazaryeri, doğrulanmadı). TR'de bulunan tek 5 mm milli 12 V 775.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Mandren / pens seti 5 mm mil</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>10 pens 0,5–3,2 mm (3,175 saplı karbür uçları tutar)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>318</v>
+      </c>
+      <c r="E8" s="3">
+        <f>IF(D8="","",C8*D8)</f>
+        <v/>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Motorobit</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>https://www.motorobit.com/el-matkabi-mandren-seti-5mm</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Var (45)</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>evet</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>JT0 yerine pens tipi. MAN02 (≤3 mm) ve MAN01 (≤2,4 mm mil) uymaz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>T8 trapez mil 400 mm + pirinç somun</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>T8x8; 150 mm'ye kesilir</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="E9" s="3">
+        <f>IF(D9="","",C9*D9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Motorobit</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>https://www.motorobit.com/3d-yazici-vidali-mil-somun-400mm-40-cm-t8-8mm</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Var (56)</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>evet</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>100–150 mm TR'de yok. Tork yetmezse T8x2 (4 kat kuvvet, 1/4 hız).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Kaplin 5x8</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Z motoru – T8</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="E10" s="3">
+        <f>IF(D10="","",C10*D10)</f>
+        <v/>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Motorobit</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>https://www.motorobit.com/aluminyum-sabit-kaplin-5x8mm</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Var (100)</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>evet</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>Esnek alt.: 84 TL (Motorobit).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Mikro switch</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>DM1-00P-130G, X/Y/Z sıfırlama</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="E11" s="3">
+        <f>IF(D11="","",C11*D11)</f>
+        <v/>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Motorobit</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>https://www.motorobit.com/dm1-00p-130g-mikro-switch</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Var</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>evet</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>12 V 3 A adaptör</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>5,5 mm jak; spindle + 5 V düşürücü girişi</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>240</v>
+      </c>
+      <c r="E12" s="3">
+        <f>IF(D12="","",C12*D12)</f>
+        <v/>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Motorobit</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>https://www.motorobit.com/12v-3a-adaptor-gs-p120300e553</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Var (58)</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>evet</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>5 V 3 A düşürücü</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>LM2596-5V; 3 x 28BYJ ~0,75 A</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>160.14</v>
+      </c>
+      <c r="E13" s="3">
+        <f>IF(D13="","",C13*D13)</f>
+        <v/>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Robotistan</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>https://www.robotistan.com/5v-3a-voltaj-regulator-karti-lm2596-5v</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Var (536)</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>evet</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>MOSFET kartı</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>15 A PWM, 3,3 V tetik (spindle)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>93.20999999999999</v>
+      </c>
+      <c r="E14" s="3">
+        <f>IF(D14="","",C14*D14)</f>
+        <v/>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Robotistan</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>https://www.robotistan.com/15a-400w-pwm-kontrollu-mosfet-anahtarlama-karti</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Var (174)</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>evet</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>+ 1N5819 diyot 1,20 TL (Motorobit).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>M3/M4 vida + somun</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Direnc paketleri (M3 16 mm, M3 somun, M4 16 mm, M4 somun)</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>92</v>
+      </c>
+      <c r="E15" s="3">
+        <f>IF(D15="","",C15*D15)</f>
+        <v/>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Direnc.net</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>https://www.direnc.net/m3-15mm-ysb-20-adet</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Var</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>hayır</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>Toplam paket fiyatı, arama verisinden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>PCB karbür uç seti</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>0,3–1,2 mm, 10 adet, 3,175 sap</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>270</v>
+      </c>
+      <c r="E16" s="3">
+        <f>IF(D16="","",C16*D16)</f>
+        <v/>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Motorobit</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>https://www.motorobit.com/pcb-matkap-ucu-seti-03-1</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Var</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>evet</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>0,6 mm altı uçlar salgıya hassas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>ESP32-S3</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Kullanıcıda var</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="3">
+        <f>IF(D17="","",C17*D17)</f>
+        <v/>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>PETG filament</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>~300 g (16 parça, %40 doluluk; kaba tahmin)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="3" t="n"/>
+      <c r="E18" s="3">
+        <f>IF(D18="","",C18*D18)</f>
+        <v/>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>hayır</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="inlineStr">
+        <is>
+          <t>Elde varsa 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Kontrplak / MDF</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Taban 370x357 (18), kolon 160x278, Z plakası 110x175, 2 yanak 105x175 (18), tabla 180x120 (9), lata 220x40 (8), feda 164x104 (3)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="3" t="n"/>
+      <c r="E19" s="3">
+        <f>IF(D19="","",C19*D19)</f>
+        <v/>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Yerel kesim</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>hayır</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>Ölçüler delme/README.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Hizalama pimi Ø3</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>DIN 6325 3x16 ya da 3 mm gümüş çelik</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="3" t="n"/>
+      <c r="E20" s="3">
+        <f>IF(D20="","",C20*D20)</f>
+        <v/>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Hırdavat</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I20" s="9" t="inlineStr">
+        <is>
+          <t>hayır</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>TR e-ticarette bulunamadı.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>TOPLAM</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr"/>
+      <c r="C21" s="4" t="inlineStr"/>
+      <c r="D21" s="5" t="inlineStr"/>
+      <c r="E21" s="5">
+        <f>SUM(E2:E20)</f>
+        <v/>
+      </c>
+      <c r="F21" s="4" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr"/>
+      <c r="H21" s="4" t="inlineStr"/>
+      <c r="I21" s="4" t="inlineStr"/>
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t>Fiyatsız satırlar hariç; kargo hariç</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5948,7 +6918,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6943,7 +7913,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7161,7 +8131,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>